<commit_message>
-- Added default option to data case argument of drop na function, required due to structure of as_flexfile, as_quantityreport class functions -- Adjusted read_maintrepair to reflect logic of TDR, properly call spec_cleanup -- Adjusted maintrepair spec in data-raw folder
</commit_message>
<xml_diff>
--- a/data-raw/maintrepair-tables.xlsx
+++ b/data-raw/maintrepair-tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25602"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ameade\Documents\M&amp;R Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bellenbogen\Software\R\readflexfile\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="74" documentId="8_{834E4B00-2B88-466B-BDBB-C78C1EF16525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37B5971C-BD7C-4054-9C3A-20A10F05A4CC}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCE6BF3D-F480-4932-889A-27E3B3932985}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" firstSheet="1" xr2:uid="{70662983-B3C8-4400-9135-830EB3B68052}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{70662983-B3C8-4400-9135-830EB3B68052}"/>
   </bookViews>
   <sheets>
     <sheet name="tables" sheetId="1" r:id="rId1"/>
@@ -176,51 +176,27 @@
     <t>commodity_type</t>
   </si>
   <si>
-    <t>ReportingOrganization/OrganizationName</t>
-  </si>
-  <si>
     <t>reporting_organization_organization_name</t>
   </si>
   <si>
-    <t>ReportingOrganization/DivisionName</t>
-  </si>
-  <si>
     <t>reporting_organization_division_name</t>
   </si>
   <si>
-    <t>ReportingOrganization/CAGECode</t>
-  </si>
-  <si>
     <t>reporting_organization_cage_code</t>
   </si>
   <si>
-    <t>ReportingOrganization/Location/Street</t>
-  </si>
-  <si>
     <t>reporting_organization_location_street</t>
   </si>
   <si>
-    <t>ReportingOrganization/Location/City</t>
-  </si>
-  <si>
     <t>reporting_organization_location_city</t>
   </si>
   <si>
-    <t>ReportingOrganization/Location/State</t>
-  </si>
-  <si>
     <t>reporting_organization_location_state</t>
   </si>
   <si>
-    <t>ReportingOrganization/Location/ZipCode</t>
-  </si>
-  <si>
     <t>reporting_organization_location_zip_code</t>
   </si>
   <si>
-    <t>ReportingOrganization/Location/Country</t>
-  </si>
-  <si>
     <t>reporting_organization_location_country</t>
   </si>
   <si>
@@ -272,18 +248,12 @@
     <t>contract_number</t>
   </si>
   <si>
-    <t>PeriodofPerformance_StartDate</t>
-  </si>
-  <si>
     <t>period_of_performance_start_date</t>
   </si>
   <si>
     <t>DATETIME</t>
   </si>
   <si>
-    <t>PeriodofPerformance_EndDate</t>
-  </si>
-  <si>
     <t>period_of_performance_end_date</t>
   </si>
   <si>
@@ -296,18 +266,12 @@
     <t>ReportCycleEnum</t>
   </si>
   <si>
-    <t>SubmissionEvent_Number</t>
-  </si>
-  <si>
     <t>submission_event_number</t>
   </si>
   <si>
     <t>LONG</t>
   </si>
   <si>
-    <t>SubmissionEvent_Name</t>
-  </si>
-  <si>
     <t>submission_event_name</t>
   </si>
   <si>
@@ -317,9 +281,6 @@
     <t>resubmission_number</t>
   </si>
   <si>
-    <t>SubmissionLot_Order</t>
-  </si>
-  <si>
     <t>submission_lot_order</t>
   </si>
   <si>
@@ -329,27 +290,15 @@
     <t>report_as_of</t>
   </si>
   <si>
-    <t>PointofContact_Name</t>
-  </si>
-  <si>
     <t>point_of_contact_name</t>
   </si>
   <si>
-    <t>PointofContact_Department</t>
-  </si>
-  <si>
     <t>point_of_contact_department</t>
   </si>
   <si>
-    <t>PointofContact_TelephoneNumber</t>
-  </si>
-  <si>
     <t>point_of_contact_telephone_number</t>
   </si>
   <si>
-    <t>PointofContact_EmailAddress</t>
-  </si>
-  <si>
     <t>point_of_contact_email_address</t>
   </si>
   <si>
@@ -392,15 +341,9 @@
     <t>maintenance_event_number</t>
   </si>
   <si>
-    <t>System/EndItemorDLRNIIN</t>
-  </si>
-  <si>
     <t>system_end_item_or_dlr_niin</t>
   </si>
   <si>
-    <t>System/EndItemSerialNumber</t>
-  </si>
-  <si>
     <t>system_end_item_serial_number</t>
   </si>
   <si>
@@ -410,15 +353,9 @@
     <t>end_item_id</t>
   </si>
   <si>
-    <t>Order/LotID</t>
-  </si>
-  <si>
     <t>order_lot_id</t>
   </si>
   <si>
-    <t>Non-MissionCapable</t>
-  </si>
-  <si>
     <t>non_mission_capable</t>
   </si>
   <si>
@@ -452,9 +389,6 @@
     <t>completion_date</t>
   </si>
   <si>
-    <t>RepairOrg/Location</t>
-  </si>
-  <si>
     <t>repair_org_location</t>
   </si>
   <si>
@@ -518,15 +452,9 @@
     <t>part_number</t>
   </si>
   <si>
-    <t>RepairPartNSN(OrNIIN)</t>
-  </si>
-  <si>
     <t>repair_part_nsn_or_niin</t>
   </si>
   <si>
-    <t>RepairPartWUC/LCN</t>
-  </si>
-  <si>
     <t>repair_part_wuc_lcn</t>
   </si>
   <si>
@@ -546,13 +474,85 @@
   </si>
   <si>
     <t>repair_cost</t>
+  </si>
+  <si>
+    <t>ReportingOrganizationOrganizationName</t>
+  </si>
+  <si>
+    <t>ReportingOrganizationDivisionName</t>
+  </si>
+  <si>
+    <t>ReportingOrganizationCAGECode</t>
+  </si>
+  <si>
+    <t>ReportingOrganizationLocationStreet</t>
+  </si>
+  <si>
+    <t>ReportingOrganizationLocationCity</t>
+  </si>
+  <si>
+    <t>ReportingOrganizationLocationState</t>
+  </si>
+  <si>
+    <t>ReportingOrganizationLocationZipCode</t>
+  </si>
+  <si>
+    <t>ReportingOrganizationLocationCountry</t>
+  </si>
+  <si>
+    <t>PeriodofPerformanceStartDate</t>
+  </si>
+  <si>
+    <t>PeriodofPerformanceEndDate</t>
+  </si>
+  <si>
+    <t>SubmissionEventNumber</t>
+  </si>
+  <si>
+    <t>SubmissionEventName</t>
+  </si>
+  <si>
+    <t>PointofContactName</t>
+  </si>
+  <si>
+    <t>PointofContactDepartment</t>
+  </si>
+  <si>
+    <t>PointofContactTelephoneNumber</t>
+  </si>
+  <si>
+    <t>PointofContactEmailAddress</t>
+  </si>
+  <si>
+    <t>SubmissionLotOrder</t>
+  </si>
+  <si>
+    <t>SystemEndItemorDLRNIIN</t>
+  </si>
+  <si>
+    <t>SystemEndItemSerialNumber</t>
+  </si>
+  <si>
+    <t>OrderLotID</t>
+  </si>
+  <si>
+    <t>NonMissionCapable</t>
+  </si>
+  <si>
+    <t>RepairPartNSNOrNIIN</t>
+  </si>
+  <si>
+    <t>RepairPartWUCLCN</t>
+  </si>
+  <si>
+    <t>RepairOrgLocation</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -589,13 +589,25 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Lucida Console"/>
+      <family val="3"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -610,7 +622,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
@@ -621,10 +633,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -643,9 +656,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -683,7 +696,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -789,7 +802,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -931,7 +944,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -940,7 +953,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F1FFA09-74B2-4371-824E-34D2F84EDB61}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.42578125" customWidth="1"/>
     <col min="2" max="2" width="18.42578125" customWidth="1"/>
@@ -948,7 +961,7 @@
     <col min="4" max="4" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -958,14 +971,14 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>5</v>
       </c>
@@ -982,7 +995,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>9</v>
       </c>
@@ -999,7 +1012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>12</v>
       </c>
@@ -1016,7 +1029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>15</v>
       </c>
@@ -1033,7 +1046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>18</v>
       </c>
@@ -1050,7 +1063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>21</v>
       </c>
@@ -1076,7 +1089,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E7621AC-F836-4EE3-904C-92EBD3C25AF5}">
   <dimension ref="A1:I73"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36.7109375" bestFit="1" customWidth="1"/>
@@ -1086,7 +1099,7 @@
     <col min="7" max="7" width="22.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1115,11 +1128,11 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="9" t="s">
         <v>31</v>
       </c>
       <c r="C2" s="6" t="s">
@@ -1138,11 +1151,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="10" t="s">
         <v>34</v>
       </c>
       <c r="C3" s="6" t="s">
@@ -1161,11 +1174,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="10" t="s">
         <v>36</v>
       </c>
       <c r="C4" s="6" t="s">
@@ -1184,11 +1197,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="10" t="s">
         <v>38</v>
       </c>
       <c r="C5" s="6" t="s">
@@ -1211,11 +1224,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="9" t="s">
         <v>42</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1234,11 +1247,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="10" t="s">
         <v>44</v>
       </c>
       <c r="C7" s="6" t="s">
@@ -1257,15 +1270,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>46</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>47</v>
       </c>
       <c r="D8" s="6"/>
       <c r="E8" s="6" t="s">
@@ -1280,15 +1293,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>48</v>
+      <c r="B9" s="10" t="s">
+        <v>147</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="6" t="s">
@@ -1303,15 +1316,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>50</v>
+      <c r="B10" s="10" t="s">
+        <v>148</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6" t="s">
@@ -1326,15 +1339,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>52</v>
+      <c r="B11" s="10" t="s">
+        <v>149</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="6" t="s">
@@ -1349,15 +1362,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>54</v>
+      <c r="B12" s="9" t="s">
+        <v>150</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6" t="s">
@@ -1372,15 +1385,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>56</v>
+      <c r="B13" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6" t="s">
@@ -1395,15 +1408,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>58</v>
+      <c r="B14" s="9" t="s">
+        <v>152</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6" t="s">
@@ -1418,15 +1431,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>60</v>
+      <c r="B15" s="9" t="s">
+        <v>153</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6" t="s">
@@ -1441,15 +1454,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>62</v>
+      <c r="B16" s="10" t="s">
+        <v>54</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6" t="s">
@@ -1464,15 +1477,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>64</v>
+      <c r="B17" s="10" t="s">
+        <v>56</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6" t="s">
@@ -1487,15 +1500,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>66</v>
+      <c r="B18" s="10" t="s">
+        <v>58</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="6" t="s">
@@ -1510,15 +1523,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>68</v>
+      <c r="B19" s="10" t="s">
+        <v>60</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="6" t="s">
@@ -1528,7 +1541,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="H19" s="6" t="s">
         <v>41</v>
@@ -1537,19 +1550,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>71</v>
+      <c r="B20" s="10" t="s">
+        <v>63</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="6" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="F20" s="6" t="b">
         <v>0</v>
@@ -1560,19 +1573,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>74</v>
+      <c r="B21" s="10" t="s">
+        <v>66</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="6" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="F21" s="6" t="b">
         <v>0</v>
@@ -1583,15 +1596,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>76</v>
+      <c r="B22" s="10" t="s">
+        <v>68</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="6" t="s">
@@ -1606,19 +1619,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>78</v>
+      <c r="B23" s="9" t="s">
+        <v>154</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="6" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="F23" s="6" t="b">
         <v>0</v>
@@ -1629,19 +1642,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>81</v>
+      <c r="B24" s="9" t="s">
+        <v>155</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="6" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="F24" s="6" t="b">
         <v>0</v>
@@ -1652,15 +1665,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>83</v>
+      <c r="B25" s="10" t="s">
+        <v>73</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6" t="s">
@@ -1670,7 +1683,7 @@
         <v>0</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>41</v>
@@ -1679,19 +1692,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>86</v>
+      <c r="B26" s="9" t="s">
+        <v>156</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>87</v>
+        <v>76</v>
       </c>
       <c r="D26" s="6"/>
       <c r="E26" s="6" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="F26" s="6" t="b">
         <v>0</v>
@@ -1702,15 +1715,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>89</v>
+      <c r="B27" s="9" t="s">
+        <v>157</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="D27" s="6"/>
       <c r="E27" s="6" t="s">
@@ -1725,19 +1738,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>91</v>
+      <c r="B28" s="9" t="s">
+        <v>79</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="D28" s="6"/>
-      <c r="E28" s="6" t="s">
-        <v>88</v>
+      <c r="E28" s="10" t="s">
+        <v>33</v>
       </c>
       <c r="F28" s="6" t="b">
         <v>0</v>
@@ -1748,15 +1761,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:9">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
         <v>5</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>93</v>
+        <v>162</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="6" t="s">
@@ -1771,19 +1784,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:9">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
         <v>5</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="D30" s="6"/>
       <c r="E30" s="6" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="F30" s="6" t="b">
         <v>0</v>
@@ -1794,15 +1807,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:9">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>97</v>
+      <c r="B31" s="9" t="s">
+        <v>158</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="D31" s="6"/>
       <c r="E31" s="6" t="s">
@@ -1817,15 +1830,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:9">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>99</v>
+      <c r="B32" s="9" t="s">
+        <v>159</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6" t="s">
@@ -1840,15 +1853,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:9">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>101</v>
+      <c r="B33" s="9" t="s">
+        <v>160</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="D33" s="6"/>
       <c r="E33" s="6" t="s">
@@ -1863,15 +1876,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>103</v>
+      <c r="B34" s="9" t="s">
+        <v>161</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="6" t="s">
@@ -1886,19 +1899,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:9">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>105</v>
+      <c r="B35" s="10" t="s">
+        <v>88</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>106</v>
+        <v>89</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="6" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="F35" s="6" t="b">
         <v>0</v>
@@ -1909,7 +1922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:9">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
         <v>9</v>
       </c>
@@ -1917,7 +1930,7 @@
         <v>41</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="6" t="s">
@@ -1927,7 +1940,7 @@
         <v>1</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>108</v>
+        <v>91</v>
       </c>
       <c r="H36" s="6" t="s">
         <v>41</v>
@@ -1936,15 +1949,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:9">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>109</v>
+        <v>92</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="6" t="s">
@@ -1959,7 +1972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:9">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="7" t="s">
         <v>12</v>
       </c>
@@ -1967,7 +1980,7 @@
         <v>41</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="6" t="s">
@@ -1986,15 +1999,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:9">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>109</v>
+        <v>92</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="6" t="s">
@@ -2009,19 +2022,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:9">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
         <v>15</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>111</v>
+        <v>94</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="D40" s="6"/>
       <c r="E40" s="6" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="F40" s="6" t="b">
         <v>0</v>
@@ -2032,7 +2045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:9">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
         <v>15</v>
       </c>
@@ -2040,7 +2053,7 @@
         <v>41</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="D41" s="6"/>
       <c r="E41" s="6" t="s">
@@ -2050,7 +2063,7 @@
         <v>0</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="H41" s="6" t="s">
         <v>41</v>
@@ -2059,15 +2072,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:9">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="7" t="s">
         <v>15</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>109</v>
+        <v>92</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="D42" s="6"/>
       <c r="E42" s="6" t="s">
@@ -2082,15 +2095,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:9">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
         <v>15</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="D43" s="6"/>
       <c r="E43" s="6" t="s">
@@ -2100,7 +2113,7 @@
         <v>0</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>113</v>
+        <v>96</v>
       </c>
       <c r="H43" s="6" t="s">
         <v>41</v>
@@ -2109,19 +2122,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:9">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="D44" s="6"/>
       <c r="E44" s="6" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="F44" s="6" t="b">
         <v>0</v>
@@ -2132,15 +2145,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:9">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>118</v>
+        <v>163</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="D45" s="6"/>
       <c r="E45" s="6" t="s">
@@ -2155,15 +2168,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:9">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>120</v>
+        <v>164</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>121</v>
+        <v>102</v>
       </c>
       <c r="D46" s="6"/>
       <c r="E46" s="6" t="s">
@@ -2178,15 +2191,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:9">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>122</v>
+        <v>103</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="D47" s="6"/>
       <c r="E47" s="6" t="s">
@@ -2205,15 +2218,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:9">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>124</v>
+        <v>165</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>125</v>
+        <v>105</v>
       </c>
       <c r="D48" s="6"/>
       <c r="E48" s="6" t="s">
@@ -2232,15 +2245,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:9">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>126</v>
+        <v>166</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>127</v>
+        <v>106</v>
       </c>
       <c r="D49" s="6"/>
       <c r="E49" s="6" t="s">
@@ -2255,15 +2268,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:9">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>128</v>
+        <v>107</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>129</v>
+        <v>108</v>
       </c>
       <c r="D50" s="6"/>
       <c r="E50" s="6" t="s">
@@ -2278,15 +2291,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:9">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>130</v>
+        <v>109</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
       <c r="D51" s="6"/>
       <c r="E51" s="6" t="s">
@@ -2301,15 +2314,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:9">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>132</v>
+        <v>111</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>133</v>
+        <v>112</v>
       </c>
       <c r="D52" s="6"/>
       <c r="E52" s="6" t="s">
@@ -2324,19 +2337,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:9">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>134</v>
+        <v>113</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>135</v>
+        <v>114</v>
       </c>
       <c r="D53" s="6"/>
       <c r="E53" s="6" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="F53" s="6" t="b">
         <v>0</v>
@@ -2347,19 +2360,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:9">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>136</v>
+        <v>115</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>137</v>
+        <v>116</v>
       </c>
       <c r="D54" s="6"/>
       <c r="E54" s="6" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="F54" s="6" t="b">
         <v>0</v>
@@ -2370,15 +2383,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:9">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>138</v>
+        <v>169</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>139</v>
+        <v>117</v>
       </c>
       <c r="D55" s="6"/>
       <c r="E55" s="6" t="s">
@@ -2393,15 +2406,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:9">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>140</v>
+        <v>118</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>141</v>
+        <v>119</v>
       </c>
       <c r="D56" s="6"/>
       <c r="E56" s="6" t="s">
@@ -2416,15 +2429,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:9">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>143</v>
+        <v>121</v>
       </c>
       <c r="D57" s="6"/>
       <c r="E57" s="6" t="s">
@@ -2439,19 +2452,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:9">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>144</v>
+        <v>122</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>145</v>
+        <v>123</v>
       </c>
       <c r="D58" s="6"/>
       <c r="E58" s="6" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="F58" s="6" t="b">
         <v>0</v>
@@ -2462,15 +2475,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:9">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
         <v>18</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>146</v>
+        <v>124</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="D59" s="6"/>
       <c r="E59" s="6" t="s">
@@ -2485,15 +2498,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:9">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="D60" s="6"/>
       <c r="E60" s="6" t="s">
@@ -2508,15 +2521,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:9">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>148</v>
+        <v>126</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>149</v>
+        <v>127</v>
       </c>
       <c r="D61" s="6"/>
       <c r="E61" s="6" t="s">
@@ -2531,15 +2544,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:9">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>150</v>
+        <v>128</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>151</v>
+        <v>129</v>
       </c>
       <c r="D62" s="6"/>
       <c r="E62" s="6" t="s">
@@ -2554,15 +2567,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:9">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>152</v>
+        <v>130</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>153</v>
+        <v>131</v>
       </c>
       <c r="D63" s="6"/>
       <c r="E63" s="6" t="s">
@@ -2577,15 +2590,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:9">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>143</v>
+        <v>121</v>
       </c>
       <c r="D64" s="6"/>
       <c r="E64" s="6" t="s">
@@ -2600,15 +2613,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:9">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>154</v>
+        <v>132</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>155</v>
+        <v>133</v>
       </c>
       <c r="D65" s="6"/>
       <c r="E65" s="6" t="s">
@@ -2623,19 +2636,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:9">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>156</v>
+        <v>134</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>157</v>
+        <v>135</v>
       </c>
       <c r="D66" s="6"/>
       <c r="E66" s="6" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="F66" s="6" t="b">
         <v>0</v>
@@ -2646,15 +2659,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:9">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>158</v>
+        <v>136</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>159</v>
+        <v>137</v>
       </c>
       <c r="D67" s="6"/>
       <c r="E67" s="6" t="s">
@@ -2669,15 +2682,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:9">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>161</v>
+        <v>138</v>
       </c>
       <c r="D68" s="6"/>
       <c r="E68" s="6" t="s">
@@ -2692,15 +2705,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:9">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>163</v>
+        <v>139</v>
       </c>
       <c r="D69" s="6"/>
       <c r="E69" s="6" t="s">
@@ -2715,15 +2728,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:9">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>164</v>
+        <v>140</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>165</v>
+        <v>141</v>
       </c>
       <c r="D70" s="6"/>
       <c r="E70" s="6" t="s">
@@ -2738,19 +2751,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:9">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>166</v>
+        <v>142</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>167</v>
+        <v>143</v>
       </c>
       <c r="D71" s="6"/>
       <c r="E71" s="6" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="F71" s="6" t="b">
         <v>0</v>
@@ -2761,19 +2774,19 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:9">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>168</v>
+        <v>144</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>169</v>
+        <v>145</v>
       </c>
       <c r="D72" s="6"/>
       <c r="E72" s="6" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="F72" s="6" t="b">
         <v>0</v>
@@ -2784,15 +2797,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:9">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
         <v>21</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>146</v>
+        <v>124</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="D73" s="6"/>
       <c r="E73" s="6" t="s">
@@ -2813,6 +2826,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CBC12096B4D56E43B1F5911C835D18E4" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="19333f2ebfefcd2362c0e88a89c5c7f8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="357ea1be-ddc3-494a-b1fb-24c1664aeba1" xmlns:ns3="22629126-c2bf-42e9-9255-22784a2ff070" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ef45f5a3df94bd17275cd31a205544ad" ns2:_="" ns3:_="">
     <xsd:import namespace="357ea1be-ddc3-494a-b1fb-24c1664aeba1"/>
@@ -3049,15 +3071,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3071,13 +3084,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A86313-FAD3-4D5A-B00F-83DBADC5A985}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37621505-38F2-4E00-8633-8E67CD5EC147}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37621505-38F2-4E00-8633-8E67CD5EC147}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A86313-FAD3-4D5A-B00F-83DBADC5A985}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="357ea1be-ddc3-494a-b1fb-24c1664aeba1"/>
+    <ds:schemaRef ds:uri="22629126-c2bf-42e9-9255-22784a2ff070"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28F795A1-B9B9-4597-B8D5-2A060002D60F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28F795A1-B9B9-4597-B8D5-2A060002D60F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="357ea1be-ddc3-494a-b1fb-24c1664aeba1"/>
+    <ds:schemaRef ds:uri="22629126-c2bf-42e9-9255-22784a2ff070"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Removed superfluous comments, added read_excel_template function, updated read_techdatareport and read_maintreport to be wrappers of read_excel_template, adjusted roxygen2 headers, adjusted spec files, wrote to news markdown file
</commit_message>
<xml_diff>
--- a/data-raw/maintrepair-tables.xlsx
+++ b/data-raw/maintrepair-tables.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ajames\Software\Git Local\costverse\readflexfile\data-raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bellenbogen\Software\R\readflexfile\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FCAC743-E26F-4E63-BB7B-FE0FC6004C09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DDBDFA5-A678-4A47-A089-F28F6BC37A9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27990" yWindow="-120" windowWidth="28110" windowHeight="16440" xr2:uid="{70662983-B3C8-4400-9135-830EB3B68052}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{70662983-B3C8-4400-9135-830EB3B68052}"/>
   </bookViews>
   <sheets>
     <sheet name="tables" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="124">
   <si>
     <t>table</t>
   </si>
@@ -257,57 +257,6 @@
     <t>RepairCost</t>
   </si>
   <si>
-    <t>ReportingOrganizationOrganizationName</t>
-  </si>
-  <si>
-    <t>ReportingOrganizationDivisionName</t>
-  </si>
-  <si>
-    <t>ReportingOrganizationCAGECode</t>
-  </si>
-  <si>
-    <t>ReportingOrganizationLocationStreet</t>
-  </si>
-  <si>
-    <t>ReportingOrganizationLocationCity</t>
-  </si>
-  <si>
-    <t>ReportingOrganizationLocationState</t>
-  </si>
-  <si>
-    <t>ReportingOrganizationLocationZipCode</t>
-  </si>
-  <si>
-    <t>ReportingOrganizationLocationCountry</t>
-  </si>
-  <si>
-    <t>PeriodofPerformanceStartDate</t>
-  </si>
-  <si>
-    <t>PeriodofPerformanceEndDate</t>
-  </si>
-  <si>
-    <t>SubmissionEventNumber</t>
-  </si>
-  <si>
-    <t>SubmissionEventName</t>
-  </si>
-  <si>
-    <t>PointofContactName</t>
-  </si>
-  <si>
-    <t>PointofContactDepartment</t>
-  </si>
-  <si>
-    <t>PointofContactTelephoneNumber</t>
-  </si>
-  <si>
-    <t>PointofContactEmailAddress</t>
-  </si>
-  <si>
-    <t>SubmissionLotOrder</t>
-  </si>
-  <si>
     <t>SystemEndItemorDLRNIIN</t>
   </si>
   <si>
@@ -405,6 +354,60 @@
   </si>
   <si>
     <t>pascal_name</t>
+  </si>
+  <si>
+    <t>PhaseOrMilestoneID</t>
+  </si>
+  <si>
+    <t>ReportingOrganization_OrganizationName</t>
+  </si>
+  <si>
+    <t>ReportingOrganization_DivisionName</t>
+  </si>
+  <si>
+    <t>ReportingOrganization_CageCode</t>
+  </si>
+  <si>
+    <t>ReportingOrganization_Location_Street</t>
+  </si>
+  <si>
+    <t>ReportingOrganization_Location_City</t>
+  </si>
+  <si>
+    <t>ReportingOrganization_Location_State</t>
+  </si>
+  <si>
+    <t>ReportingOrganization_Location_ZipCode</t>
+  </si>
+  <si>
+    <t>ReportingOrganization_Location_Country</t>
+  </si>
+  <si>
+    <t>PeriodOfPerformance_StartDate</t>
+  </si>
+  <si>
+    <t>PeriodOfPerformance_EndDate</t>
+  </si>
+  <si>
+    <t>SubmissionEvent_Number</t>
+  </si>
+  <si>
+    <t>SubmissionEvent_Name</t>
+  </si>
+  <si>
+    <t>PointOfContact_Name</t>
+  </si>
+  <si>
+    <t>PointOfContact_Department</t>
+  </si>
+  <si>
+    <t>PointOfContact_TelephoneNumber</t>
+  </si>
+  <si>
+    <t>PointOfContact_EmailAddress</t>
+  </si>
+  <si>
+    <t>SubmissionLot_Order</t>
   </si>
 </sst>
 </file>
@@ -450,7 +453,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -460,6 +463,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -476,7 +485,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -489,6 +498,8 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -820,7 +831,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>2</v>
@@ -960,7 +971,7 @@
         <v>17</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>18</v>
@@ -988,7 +999,7 @@
       <c r="B2" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>23</v>
       </c>
       <c r="E2" s="4" t="s">
@@ -1008,7 +1019,7 @@
       <c r="B3" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="4" t="s">
         <v>25</v>
       </c>
       <c r="E3" s="4" t="s">
@@ -1028,7 +1039,7 @@
       <c r="B4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="4" t="s">
         <v>26</v>
       </c>
       <c r="E4" s="4" t="s">
@@ -1048,8 +1059,8 @@
       <c r="B5" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>27</v>
+      <c r="C5" s="4" t="s">
+        <v>106</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>24</v>
@@ -1074,7 +1085,7 @@
       <c r="B6" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>30</v>
       </c>
       <c r="E6" s="4" t="s">
@@ -1094,7 +1105,7 @@
       <c r="B7" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="4" t="s">
         <v>31</v>
       </c>
       <c r="E7" s="4" t="s">
@@ -1112,10 +1123,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>73</v>
+        <v>80</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>107</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>24</v>
@@ -1132,10 +1143,10 @@
         <v>4</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>74</v>
+        <v>81</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>108</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>24</v>
@@ -1152,10 +1163,10 @@
         <v>4</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>75</v>
+        <v>82</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>109</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>24</v>
@@ -1172,10 +1183,10 @@
         <v>4</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>76</v>
+        <v>83</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>110</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>24</v>
@@ -1192,10 +1203,10 @@
         <v>4</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>77</v>
+        <v>84</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>111</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>24</v>
@@ -1212,10 +1223,10 @@
         <v>4</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>78</v>
+        <v>85</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>112</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>24</v>
@@ -1232,10 +1243,10 @@
         <v>4</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>79</v>
+        <v>86</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>113</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>24</v>
@@ -1252,10 +1263,10 @@
         <v>4</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>80</v>
+        <v>87</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>114</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>24</v>
@@ -1274,7 +1285,7 @@
       <c r="B16" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="4" t="s">
         <v>32</v>
       </c>
       <c r="E16" s="4" t="s">
@@ -1294,7 +1305,7 @@
       <c r="B17" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="4" t="s">
         <v>33</v>
       </c>
       <c r="E17" s="4" t="s">
@@ -1314,7 +1325,7 @@
       <c r="B18" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="4" t="s">
         <v>34</v>
       </c>
       <c r="E18" s="4" t="s">
@@ -1334,7 +1345,7 @@
       <c r="B19" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="4" t="s">
         <v>35</v>
       </c>
       <c r="E19" s="4" t="s">
@@ -1360,7 +1371,7 @@
       <c r="B20" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="4" t="s">
         <v>37</v>
       </c>
       <c r="E20" s="4" t="s">
@@ -1380,7 +1391,7 @@
       <c r="B21" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="4" t="s">
         <v>39</v>
       </c>
       <c r="E21" s="4" t="s">
@@ -1400,7 +1411,7 @@
       <c r="B22" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="4" t="s">
         <v>40</v>
       </c>
       <c r="E22" s="4" t="s">
@@ -1418,10 +1429,10 @@
         <v>4</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>81</v>
+        <v>88</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>115</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>41</v>
@@ -1438,10 +1449,10 @@
         <v>4</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>82</v>
+        <v>89</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>116</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>41</v>
@@ -1460,7 +1471,7 @@
       <c r="B25" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="4" t="s">
         <v>42</v>
       </c>
       <c r="E25" s="4" t="s">
@@ -1484,10 +1495,10 @@
         <v>4</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>83</v>
+        <v>90</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>117</v>
       </c>
       <c r="E26" s="4" t="s">
         <v>44</v>
@@ -1504,10 +1515,10 @@
         <v>4</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>84</v>
+        <v>91</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>118</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>24</v>
@@ -1526,7 +1537,7 @@
       <c r="B28" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="4" t="s">
         <v>45</v>
       </c>
       <c r="E28" s="6" t="s">
@@ -1544,10 +1555,10 @@
         <v>4</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>89</v>
+        <v>92</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>123</v>
       </c>
       <c r="E29" s="4" t="s">
         <v>24</v>
@@ -1566,7 +1577,7 @@
       <c r="B30" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="8" t="s">
         <v>46</v>
       </c>
       <c r="E30" s="4" t="s">
@@ -1584,10 +1595,10 @@
         <v>4</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>85</v>
+        <v>93</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>119</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>24</v>
@@ -1604,10 +1615,10 @@
         <v>4</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>86</v>
+        <v>94</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>120</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>24</v>
@@ -1624,10 +1635,10 @@
         <v>4</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>87</v>
+        <v>95</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>121</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>24</v>
@@ -1644,10 +1655,10 @@
         <v>4</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>88</v>
+        <v>96</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>122</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>24</v>
@@ -1666,7 +1677,7 @@
       <c r="B35" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="C35" s="4" t="s">
         <v>47</v>
       </c>
       <c r="E35" s="4" t="s">
@@ -1888,10 +1899,10 @@
         <v>13</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>24</v>
@@ -1908,10 +1919,10 @@
         <v>13</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>115</v>
+        <v>98</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="E46" s="4" t="s">
         <v>24</v>
@@ -1954,10 +1965,10 @@
         <v>13</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="E48" s="4" t="s">
         <v>24</v>
@@ -1980,10 +1991,10 @@
         <v>13</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="E49" s="4" t="s">
         <v>24</v>
@@ -2100,10 +2111,10 @@
         <v>13</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>118</v>
+        <v>101</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="E55" s="4" t="s">
         <v>24</v>
@@ -2360,10 +2371,10 @@
         <v>15</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="E68" s="4" t="s">
         <v>24</v>
@@ -2380,10 +2391,10 @@
         <v>15</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>120</v>
+        <v>103</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="E69" s="4" t="s">
         <v>24</v>
@@ -2493,6 +2504,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CBC12096B4D56E43B1F5911C835D18E4" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="19333f2ebfefcd2362c0e88a89c5c7f8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="357ea1be-ddc3-494a-b1fb-24c1664aeba1" xmlns:ns3="22629126-c2bf-42e9-9255-22784a2ff070" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ef45f5a3df94bd17275cd31a205544ad" ns2:_="" ns3:_="">
     <xsd:import namespace="357ea1be-ddc3-494a-b1fb-24c1664aeba1"/>
@@ -2729,15 +2749,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28F795A1-B9B9-4597-B8D5-2A060002D60F}">
   <ds:schemaRefs>
@@ -2750,6 +2761,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37621505-38F2-4E00-8633-8E67CD5EC147}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{67A86313-FAD3-4D5A-B00F-83DBADC5A985}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2766,12 +2785,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{37621505-38F2-4E00-8633-8E67CD5EC147}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>